<commit_message>
Add Ashik-PC (AST-0047) to Endpoints
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/company_assets_sample.xlsx
+++ b/company_assets_sample.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Registers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Endpoints'!$A$1:$S$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Endpoints'!$A$1:$S$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Servers'!$A$1:$S$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Registers'!$A$1:$I$21</definedName>
   </definedNames>
@@ -1955,7 +1955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="27" min="1" max="1"/>
@@ -6260,8 +6260,55 @@
         <v>46307</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="32" t="inlineStr">
+        <is>
+          <t>AST-0047</t>
+        </is>
+      </c>
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>Ashik-PC</t>
+        </is>
+      </c>
+      <c r="C48" s="32" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D48" s="32" t="inlineStr">
+        <is>
+          <t>macOS</t>
+        </is>
+      </c>
+      <c r="E48" s="32" t="n"/>
+      <c r="F48" s="32" t="n"/>
+      <c r="G48" s="32" t="n"/>
+      <c r="H48" s="32" t="n"/>
+      <c r="I48" s="32" t="n"/>
+      <c r="J48" s="32" t="n"/>
+      <c r="K48" s="32" t="n"/>
+      <c r="L48" s="32" t="n"/>
+      <c r="M48" s="32" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N48" s="37" t="n"/>
+      <c r="O48" s="37" t="n"/>
+      <c r="P48" s="32" t="inlineStr">
+        <is>
+          <t>CrowdStrike Falcon</t>
+        </is>
+      </c>
+      <c r="Q48" s="32" t="n"/>
+      <c r="R48" s="32" t="n"/>
+      <c r="S48" s="37" t="n">
+        <v>46307</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S47"/>
+  <autoFilter ref="A1:S48"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>